<commit_message>
Update index: 17046 → 17047 [scan complete]
Scanned address נובומיסקי משה 1 (index 17046).
Found 1 business: גל יהודה, מחשבים (נובומיסקי משה 1/2).
Token budget reached (30,000 tokens). Stopping scan.
Excel report generated for 2026-09-10.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YGNCPy7oyb5iygmuKxzCfu
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:10-09-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:10-09-2026.xlsx
@@ -26,15 +26,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -47,17 +44,15 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -65,16 +60,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="001F4E79"/>
+      </left>
+      <right style="thin">
+        <color rgb="001F4E79"/>
+      </right>
+      <top style="thin">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001F4E79"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,17 +454,17 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>שם העסק</t>
@@ -495,17 +506,37 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>סריקה: נהר פרת 9 ירושלים — לא נמצאו עסקים מאומתים בכתובת זו</t>
-        </is>
-      </c>
+          <t>גל יהודה, מחשבים</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>נובומיסקי משה 1/2, ירושלים 9690801</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>מחשבים / ציוד טכנולוגי</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dunsguide.co.il/Ca952a9f1814433f8ac2e44331205e43d_%D7%97%D7%91%D7%A8%D7%95%D7%AA_%D7%94%D7%99%D7%99%D7%98%D7%A7_%D7%95%D7%9E%D7%99%D7%97%D7%A9%D7%95%D7%91/%D7%92%D7%9C%D7%A8%D7%99_%D7%9E%D7%97%D7%A9%D7%91%D7%99%D7%9D</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:H2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>